<commit_message>
polar ae shop trial
</commit_message>
<xml_diff>
--- a/Aepms-backend/data/ae_shop_trial.xlsx
+++ b/Aepms-backend/data/ae_shop_trial.xlsx
@@ -8,20 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GOKUL\Desktop\WORKPLACE\Workplace\Aepms-backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A389AF-6726-4A53-A5E7-821C3412C7DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63EC472-835E-44F8-8BC4-35973ECF1C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vessel_generators" sheetId="1" r:id="rId1"/>
     <sheet name="generator_baseline_data" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="64">
   <si>
     <t>imo_number</t>
   </si>
@@ -195,6 +206,24 @@
   </si>
   <si>
     <t>1764FXJ</t>
+  </si>
+  <si>
+    <t>PAAE161795</t>
+  </si>
+  <si>
+    <t>PAAE161794</t>
+  </si>
+  <si>
+    <t>PAAE161793</t>
+  </si>
+  <si>
+    <t>WARTSILA</t>
+  </si>
+  <si>
+    <t>A4L20</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -660,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.77734375" customWidth="1"/>
@@ -1635,6 +1664,84 @@
         <v>900</v>
       </c>
     </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>9521813</v>
+      </c>
+      <c r="B38" t="s">
+        <v>58</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" t="s">
+        <v>61</v>
+      </c>
+      <c r="E38" t="s">
+        <v>62</v>
+      </c>
+      <c r="F38">
+        <v>4</v>
+      </c>
+      <c r="G38">
+        <v>548</v>
+      </c>
+      <c r="H38">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>9521813</v>
+      </c>
+      <c r="B39" t="s">
+        <v>59</v>
+      </c>
+      <c r="C39" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" t="s">
+        <v>61</v>
+      </c>
+      <c r="E39" t="s">
+        <v>62</v>
+      </c>
+      <c r="F39">
+        <v>4</v>
+      </c>
+      <c r="G39">
+        <v>548</v>
+      </c>
+      <c r="H39">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>9521813</v>
+      </c>
+      <c r="B40" t="s">
+        <v>60</v>
+      </c>
+      <c r="C40" t="s">
+        <v>12</v>
+      </c>
+      <c r="D40" t="s">
+        <v>61</v>
+      </c>
+      <c r="E40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F40">
+        <v>4</v>
+      </c>
+      <c r="G40">
+        <v>680</v>
+      </c>
+      <c r="H40">
+        <v>900</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1646,7 +1753,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K181"/>
+  <dimension ref="A1:K199"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="13.33203125" customWidth="1"/>
@@ -7924,6 +8031,636 @@
         <v>205.19</v>
       </c>
     </row>
+    <row r="182" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A182">
+        <v>9521813</v>
+      </c>
+      <c r="B182" t="s">
+        <v>58</v>
+      </c>
+      <c r="C182">
+        <v>25</v>
+      </c>
+      <c r="D182">
+        <v>139</v>
+      </c>
+      <c r="E182" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F182" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G182" t="s">
+        <v>53</v>
+      </c>
+      <c r="H182" s="3">
+        <v>321</v>
+      </c>
+      <c r="I182" s="3">
+        <v>319</v>
+      </c>
+      <c r="J182" s="3">
+        <v>12</v>
+      </c>
+      <c r="K182" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="183" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A183">
+        <v>9521813</v>
+      </c>
+      <c r="B183" t="s">
+        <v>58</v>
+      </c>
+      <c r="C183">
+        <v>50</v>
+      </c>
+      <c r="D183">
+        <v>273</v>
+      </c>
+      <c r="E183" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F183" s="3">
+        <v>1</v>
+      </c>
+      <c r="G183" t="s">
+        <v>53</v>
+      </c>
+      <c r="H183" s="3">
+        <v>342</v>
+      </c>
+      <c r="I183" s="3">
+        <v>344</v>
+      </c>
+      <c r="J183" s="3">
+        <v>16</v>
+      </c>
+      <c r="K183" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="184" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A184">
+        <v>9521813</v>
+      </c>
+      <c r="B184" t="s">
+        <v>58</v>
+      </c>
+      <c r="C184">
+        <v>75</v>
+      </c>
+      <c r="D184">
+        <v>408</v>
+      </c>
+      <c r="E184" s="3">
+        <v>12.8</v>
+      </c>
+      <c r="F184" s="3">
+        <v>1.7</v>
+      </c>
+      <c r="G184" t="s">
+        <v>53</v>
+      </c>
+      <c r="H184" s="3">
+        <v>360</v>
+      </c>
+      <c r="I184" s="3">
+        <v>331</v>
+      </c>
+      <c r="J184" s="3">
+        <v>21</v>
+      </c>
+      <c r="K184" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="185" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A185">
+        <v>9521813</v>
+      </c>
+      <c r="B185" t="s">
+        <v>58</v>
+      </c>
+      <c r="C185">
+        <v>85</v>
+      </c>
+      <c r="D185">
+        <v>462</v>
+      </c>
+      <c r="E185" s="3">
+        <v>13.9</v>
+      </c>
+      <c r="F185" s="3">
+        <v>2</v>
+      </c>
+      <c r="G185" t="s">
+        <v>53</v>
+      </c>
+      <c r="H185" s="3">
+        <v>370</v>
+      </c>
+      <c r="I185" s="3">
+        <v>333</v>
+      </c>
+      <c r="J185" s="3">
+        <v>22</v>
+      </c>
+      <c r="K185" s="3">
+        <v>205.4</v>
+      </c>
+    </row>
+    <row r="186" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A186">
+        <v>9521813</v>
+      </c>
+      <c r="B186" t="s">
+        <v>58</v>
+      </c>
+      <c r="C186">
+        <v>100</v>
+      </c>
+      <c r="D186">
+        <v>545</v>
+      </c>
+      <c r="E186" s="3">
+        <v>15.5</v>
+      </c>
+      <c r="F186" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="G186" t="s">
+        <v>53</v>
+      </c>
+      <c r="H186" s="3">
+        <v>385</v>
+      </c>
+      <c r="I186" s="3">
+        <v>330</v>
+      </c>
+      <c r="J186" s="3">
+        <v>24</v>
+      </c>
+      <c r="K186" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="187" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A187">
+        <v>9521813</v>
+      </c>
+      <c r="B187" t="s">
+        <v>58</v>
+      </c>
+      <c r="C187">
+        <v>110</v>
+      </c>
+      <c r="D187">
+        <v>599</v>
+      </c>
+      <c r="E187" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F187" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="G187" t="s">
+        <v>53</v>
+      </c>
+      <c r="H187" s="3">
+        <v>394</v>
+      </c>
+      <c r="I187" s="3">
+        <v>326</v>
+      </c>
+      <c r="J187" s="3">
+        <v>26</v>
+      </c>
+      <c r="K187" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="188" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A188">
+        <v>9521813</v>
+      </c>
+      <c r="B188" t="s">
+        <v>59</v>
+      </c>
+      <c r="C188">
+        <v>25</v>
+      </c>
+      <c r="D188">
+        <v>139</v>
+      </c>
+      <c r="E188" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F188" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="G188" t="s">
+        <v>53</v>
+      </c>
+      <c r="H188" s="3">
+        <v>316</v>
+      </c>
+      <c r="I188" s="3">
+        <v>332</v>
+      </c>
+      <c r="J188" s="3">
+        <v>12</v>
+      </c>
+      <c r="K188" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="189" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A189">
+        <v>9521813</v>
+      </c>
+      <c r="B189" t="s">
+        <v>59</v>
+      </c>
+      <c r="C189">
+        <v>50</v>
+      </c>
+      <c r="D189">
+        <v>273</v>
+      </c>
+      <c r="E189" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F189" s="3">
+        <v>1</v>
+      </c>
+      <c r="G189" t="s">
+        <v>53</v>
+      </c>
+      <c r="H189" s="3">
+        <v>339</v>
+      </c>
+      <c r="I189" s="3">
+        <v>350</v>
+      </c>
+      <c r="J189" s="3">
+        <v>16.5</v>
+      </c>
+      <c r="K189" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="190" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A190">
+        <v>9521813</v>
+      </c>
+      <c r="B190" t="s">
+        <v>59</v>
+      </c>
+      <c r="C190">
+        <v>75</v>
+      </c>
+      <c r="D190">
+        <v>408</v>
+      </c>
+      <c r="E190" s="3">
+        <v>12.9</v>
+      </c>
+      <c r="F190" s="3">
+        <v>1.7</v>
+      </c>
+      <c r="G190" t="s">
+        <v>53</v>
+      </c>
+      <c r="H190" s="3">
+        <v>360</v>
+      </c>
+      <c r="I190" s="3">
+        <v>340</v>
+      </c>
+      <c r="J190" s="3">
+        <v>21</v>
+      </c>
+      <c r="K190" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="191" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A191">
+        <v>9521813</v>
+      </c>
+      <c r="B191" t="s">
+        <v>59</v>
+      </c>
+      <c r="C191">
+        <v>85</v>
+      </c>
+      <c r="D191">
+        <v>462</v>
+      </c>
+      <c r="E191" s="3">
+        <v>14.2</v>
+      </c>
+      <c r="F191" s="3">
+        <v>1.9</v>
+      </c>
+      <c r="G191" t="s">
+        <v>53</v>
+      </c>
+      <c r="H191" s="3">
+        <v>369</v>
+      </c>
+      <c r="I191" s="3">
+        <v>339</v>
+      </c>
+      <c r="J191" s="3">
+        <v>22</v>
+      </c>
+      <c r="K191" s="3">
+        <v>191.6</v>
+      </c>
+    </row>
+    <row r="192" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A192">
+        <v>9521813</v>
+      </c>
+      <c r="B192" t="s">
+        <v>59</v>
+      </c>
+      <c r="C192">
+        <v>100</v>
+      </c>
+      <c r="D192">
+        <v>545</v>
+      </c>
+      <c r="E192" s="3">
+        <v>15.6</v>
+      </c>
+      <c r="F192" s="3">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="G192" t="s">
+        <v>53</v>
+      </c>
+      <c r="H192" s="3">
+        <v>381</v>
+      </c>
+      <c r="I192" s="3">
+        <v>335</v>
+      </c>
+      <c r="J192" s="3">
+        <v>24</v>
+      </c>
+      <c r="K192" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="193" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A193">
+        <v>9521813</v>
+      </c>
+      <c r="B193" t="s">
+        <v>59</v>
+      </c>
+      <c r="C193">
+        <v>110</v>
+      </c>
+      <c r="D193">
+        <v>599</v>
+      </c>
+      <c r="E193" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F193" s="3">
+        <v>2.6</v>
+      </c>
+      <c r="G193" t="s">
+        <v>53</v>
+      </c>
+      <c r="H193" s="3">
+        <v>389</v>
+      </c>
+      <c r="I193" s="3">
+        <v>327</v>
+      </c>
+      <c r="J193" s="3">
+        <v>26</v>
+      </c>
+      <c r="K193" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="194" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A194">
+        <v>9521813</v>
+      </c>
+      <c r="B194" t="s">
+        <v>60</v>
+      </c>
+      <c r="C194">
+        <v>25</v>
+      </c>
+      <c r="D194">
+        <v>173</v>
+      </c>
+      <c r="E194" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F194" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="G194" t="s">
+        <v>53</v>
+      </c>
+      <c r="H194" s="3">
+        <v>317</v>
+      </c>
+      <c r="I194" s="3">
+        <v>327</v>
+      </c>
+      <c r="J194" s="3">
+        <v>13</v>
+      </c>
+      <c r="K194" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="195" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A195">
+        <v>9521813</v>
+      </c>
+      <c r="B195" t="s">
+        <v>60</v>
+      </c>
+      <c r="C195">
+        <v>50</v>
+      </c>
+      <c r="D195">
+        <v>337</v>
+      </c>
+      <c r="E195" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F195" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="G195" t="s">
+        <v>53</v>
+      </c>
+      <c r="H195" s="3">
+        <v>342</v>
+      </c>
+      <c r="I195" s="3">
+        <v>336</v>
+      </c>
+      <c r="J195" s="3">
+        <v>19</v>
+      </c>
+      <c r="K195" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="196" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A196">
+        <v>9521813</v>
+      </c>
+      <c r="B196" t="s">
+        <v>60</v>
+      </c>
+      <c r="C196">
+        <v>75</v>
+      </c>
+      <c r="D196">
+        <v>504</v>
+      </c>
+      <c r="E196" s="3">
+        <v>14.5</v>
+      </c>
+      <c r="F196" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G196" t="s">
+        <v>53</v>
+      </c>
+      <c r="H196" s="3">
+        <v>360</v>
+      </c>
+      <c r="I196" s="3">
+        <v>316</v>
+      </c>
+      <c r="J196" s="3">
+        <v>24</v>
+      </c>
+      <c r="K196" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="197" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A197">
+        <v>9521813</v>
+      </c>
+      <c r="B197" t="s">
+        <v>60</v>
+      </c>
+      <c r="C197">
+        <v>85</v>
+      </c>
+      <c r="D197">
+        <v>570</v>
+      </c>
+      <c r="E197" s="3">
+        <v>15.9</v>
+      </c>
+      <c r="F197" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="G197" t="s">
+        <v>53</v>
+      </c>
+      <c r="H197" s="3">
+        <v>373</v>
+      </c>
+      <c r="I197" s="3">
+        <v>318</v>
+      </c>
+      <c r="J197" s="3">
+        <v>15</v>
+      </c>
+      <c r="K197" s="3">
+        <v>207.4</v>
+      </c>
+    </row>
+    <row r="198" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A198">
+        <v>9521813</v>
+      </c>
+      <c r="B198" t="s">
+        <v>60</v>
+      </c>
+      <c r="C198">
+        <v>100</v>
+      </c>
+      <c r="D198">
+        <v>671</v>
+      </c>
+      <c r="E198" s="3">
+        <v>17.3</v>
+      </c>
+      <c r="F198" s="3">
+        <v>3</v>
+      </c>
+      <c r="G198" t="s">
+        <v>53</v>
+      </c>
+      <c r="H198" s="3">
+        <v>394</v>
+      </c>
+      <c r="I198" s="3">
+        <v>319</v>
+      </c>
+      <c r="J198" s="3">
+        <v>28</v>
+      </c>
+      <c r="K198" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="199" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A199">
+        <v>9521813</v>
+      </c>
+      <c r="B199" t="s">
+        <v>60</v>
+      </c>
+      <c r="C199">
+        <v>110</v>
+      </c>
+      <c r="D199">
+        <v>743</v>
+      </c>
+      <c r="E199" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F199" s="3">
+        <v>3.4</v>
+      </c>
+      <c r="G199" t="s">
+        <v>53</v>
+      </c>
+      <c r="H199" s="3">
+        <v>409</v>
+      </c>
+      <c r="I199" s="3">
+        <v>321</v>
+      </c>
+      <c r="J199" s="3">
+        <v>31</v>
+      </c>
+      <c r="K199" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>